<commit_message>
Update code on 17 feb
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14790" windowHeight="3450" firstSheet="9" activeTab="12"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14745" windowHeight="4485" firstSheet="19" activeTab="21"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="Templates" sheetId="44" r:id="rId22"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:E9"/>
+  <oleSize ref="A1:K12"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="199">
   <si>
     <t>Username</t>
   </si>
@@ -648,13 +648,10 @@
     <t>cvnamed</t>
   </si>
   <si>
-    <t>demoserver.demoroom</t>
-  </si>
-  <si>
-    <t>http://10.4.8.10:8080/CVWeb/cvLgn</t>
-  </si>
-  <si>
-    <t>Dipak_sql_Room.test_sql_room</t>
+    <t>http://10.4.10.167:8080/CVWeb/cvLgn</t>
+  </si>
+  <si>
+    <t>Win2025_Server.CV2026_Win2025_Demo</t>
   </si>
 </sst>
 </file>
@@ -1228,7 +1225,7 @@
         <v>195</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1239,7 +1236,7 @@
         <v>195</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1250,7 +1247,7 @@
         <v>195</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1630,7 +1627,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="5" customWidth="1"/>
@@ -1671,10 +1668,10 @@
         <v>195</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E2" s="6">
         <v>10</v>
@@ -1706,6 +1703,7 @@
     <hyperlink ref="B2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2588,7 +2586,7 @@
         <v>195</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2599,7 +2597,7 @@
         <v>195</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2608,7 +2606,7 @@
         <v>195</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2617,7 +2615,7 @@
       </c>
       <c r="B5" s="40"/>
       <c r="C5" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2756,7 +2754,7 @@
         <v>195</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:3">

</xml_diff>

<commit_message>
Code Added on 05 june 2026
</commit_message>
<xml_diff>
--- a/data/TestData.xlsx
+++ b/data/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14745" windowHeight="4485" firstSheet="19" activeTab="21"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13980" windowHeight="3555"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="Templates" sheetId="44" r:id="rId22"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:K12"/>
+  <oleSize ref="A1:I6"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="207">
   <si>
     <t>Username</t>
   </si>
@@ -169,9 +169,6 @@
   </si>
   <si>
     <t>Vidya</t>
-  </si>
-  <si>
-    <t>Dipak</t>
   </si>
   <si>
     <t>This is End Workflow comments</t>
@@ -648,22 +645,56 @@
     <t>cvnamed</t>
   </si>
   <si>
-    <t>http://10.4.10.167:8080/CVWeb/cvLgn</t>
-  </si>
-  <si>
     <t>Win2025_Server.CV2026_Win2025_Demo</t>
+  </si>
+  <si>
+    <t>http://13.204.55.55:8080/CVWeb/cvLgn</t>
+  </si>
+  <si>
+    <t>SERVER.ORA_ROOM1</t>
+  </si>
+  <si>
+    <t>Admin@123</t>
+  </si>
+  <si>
+    <t>cvadmin</t>
+  </si>
+  <si>
+    <t>cvuser1</t>
+  </si>
+  <si>
+    <t>Admin@125</t>
+  </si>
+  <si>
+    <t>Admin@126</t>
+  </si>
+  <si>
+    <t>Admin@127</t>
+  </si>
+  <si>
+    <t>Admin@128</t>
+  </si>
+  <si>
+    <t>Admin@129</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -834,18 +865,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
@@ -856,72 +887,76 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1219,82 +1254,78 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="35" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>195</v>
+        <v>107</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>199</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="35" t="s">
-        <v>108</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>195</v>
+        <v>107</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>199</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>195</v>
+      <c r="A4" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>202</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>195</v>
+        <v>63</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>203</v>
       </c>
       <c r="C5" s="1"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>195</v>
+        <v>183</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>195</v>
+        <v>184</v>
+      </c>
+      <c r="B7" s="42" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>195</v>
+      <c r="B8" s="42" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1"/>
-    <hyperlink ref="B3" r:id="rId2"/>
-    <hyperlink ref="B4" r:id="rId3"/>
-    <hyperlink ref="B5" r:id="rId4"/>
-    <hyperlink ref="B6" r:id="rId5"/>
-    <hyperlink ref="B7" r:id="rId6"/>
-    <hyperlink ref="B8" r:id="rId7"/>
+    <hyperlink ref="B3:B8" r:id="rId2" display="Admin@123"/>
+    <hyperlink ref="B3" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
@@ -1339,55 +1370,55 @@
         <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="D3" t="s">
-        <v>46</v>
-      </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D4" t="s">
         <v>106</v>
       </c>
-      <c r="D4" t="s">
-        <v>107</v>
-      </c>
       <c r="E4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1446,94 +1477,94 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" t="s">
         <v>41</v>
-      </c>
-      <c r="H2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F3" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>50</v>
-      </c>
-      <c r="G3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="60">
       <c r="A4" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="60">
       <c r="A5" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" t="s">
         <v>110</v>
       </c>
-      <c r="B5" t="s">
-        <v>111</v>
-      </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="B7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" t="s">
         <v>118</v>
-      </c>
-      <c r="B8" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1559,29 +1590,29 @@
   <sheetData>
     <row r="1" spans="1:5" ht="180">
       <c r="A1" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
         <v>126</v>
-      </c>
-      <c r="B2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1589,35 +1620,35 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="B5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="17" customFormat="1">
       <c r="A6" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="C6" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="D6" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="E6" s="17" t="s">
         <v>182</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -1627,7 +1658,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="5" customWidth="1"/>
@@ -1648,29 +1679,29 @@
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E1" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="F1" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="F1" s="18" t="s">
-        <v>169</v>
-      </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C2" s="22" t="s">
+      <c r="A2" s="43" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="42" t="s">
         <v>197</v>
       </c>
       <c r="E2" s="6">
@@ -1681,8 +1712,8 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="23" t="s">
-        <v>64</v>
+      <c r="A3" s="43" t="s">
+        <v>201</v>
       </c>
       <c r="B3" s="19"/>
       <c r="E3" s="6">
@@ -1700,10 +1731,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1727,24 +1759,24 @@
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D1" s="11" t="s">
         <v>170</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1776,30 +1808,30 @@
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D1" s="12" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1808,13 +1840,13 @@
         <v>4</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="19"/>
       <c r="E4" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1846,10 +1878,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="14" t="s">
         <v>173</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>174</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>17</v>
@@ -1857,19 +1889,19 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1878,10 +1910,10 @@
         <v>4</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E3" s="5"/>
     </row>
@@ -1889,10 +1921,10 @@
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E4" s="5"/>
     </row>
@@ -1900,10 +1932,10 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E5" s="5"/>
     </row>
@@ -1911,10 +1943,10 @@
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E6" s="5"/>
     </row>
@@ -1922,10 +1954,10 @@
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E7" s="5"/>
     </row>
@@ -1933,10 +1965,10 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E8" s="5"/>
     </row>
@@ -1944,7 +1976,7 @@
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -1953,7 +1985,7 @@
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -1962,7 +1994,7 @@
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -1971,7 +2003,7 @@
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -2007,30 +2039,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="37" t="s">
-        <v>195</v>
+      <c r="A2" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="39" t="s">
-        <v>196</v>
+      <c r="A5" s="38" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2052,17 +2084,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:1">
@@ -2072,7 +2104,7 @@
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2091,42 +2123,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="21" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="27" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="22" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="28" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="30" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:1">
@@ -2141,17 +2173,17 @@
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -2161,42 +2193,42 @@
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="32" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="32" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="33" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="32" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" s="32" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2215,23 +2247,23 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2239,38 +2271,38 @@
         <v>9966881234</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="C7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="C8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="C9" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2289,102 +2321,102 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:1">
@@ -2406,22 +2438,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="22" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="22" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2440,42 +2472,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2495,58 +2527,58 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" t="s">
         <v>153</v>
-      </c>
-      <c r="B1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2568,54 +2600,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="39" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="41" t="s">
-        <v>195</v>
+      <c r="A2" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="40" t="s">
+        <v>194</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="B3" s="41" t="s">
-        <v>195</v>
+      <c r="A3" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>194</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="40"/>
-      <c r="B4" s="41" t="s">
-        <v>195</v>
+      <c r="A4" s="39"/>
+      <c r="B4" s="40" t="s">
+        <v>194</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="B5" s="40"/>
+      <c r="A5" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="39"/>
       <c r="C5" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -2747,14 +2779,14 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>195</v>
+      <c r="A2" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>199</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2790,12 +2822,12 @@
         <v>19</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
         <v>20</v>
@@ -2804,39 +2836,39 @@
         <v>21</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" t="s">
         <v>63</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="C4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="D5" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="D6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>